<commit_message>
Stage 8 review fixes: B-023
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2020/BW20_0137/Run_sheets/BW20_0137_RUN04.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2020/BW20_0137/Run_sheets/BW20_0137_RUN04.xlsx
@@ -178,7 +178,7 @@
   <commentList>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Client name as it stood on the 2020 quote. Rennelwick has not been renamed on this project.</t>
+        <t>Test-lot and sample handling details remain on the original sample cards.</t>
       </text>
     </comment>
   </commentList>
@@ -188,12 +188,12 @@
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Ravi Deshmukh</author>
+    <author>Ines Alvarado</author>
   </authors>
   <commentList>
-    <comment ref="G4" authorId="0" shapeId="0">
+    <comment ref="C3" authorId="0" shapeId="0">
       <text>
-        <t>Recovery on RED-01 was the reason for the repeat. The first read is kept so the rerun is traceable.</t>
+        <t>Use the original recovery record for the dialysis run; no repeat history is assigned here.</t>
       </text>
     </comment>
   </commentList>
@@ -208,7 +208,7 @@
   <commentList>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>Recovery column is the check that the repeat worked. Anything under 80 would have been a rerun.</t>
+        <t>Consult the original dialysis run sheets for recovery acceptance and any sample-specific qualification.</t>
       </text>
     </comment>
   </commentList>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -619,7 +619,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Liver microsomal stability; plasma protein binding (RED)</t>
+          <t>HLM/RLM stability; RED PPB</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Study stage</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -637,19 +637,14 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Checked by</t>
+          <t>Record</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Microsome run</t>
+          <t>Interim</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -659,85 +654,47 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Human and rat CLint, t½</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>I. Alvarado</t>
+          <t>Study interim</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>RED run, first</t>
+          <t>Completion</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>29/04/2020</t>
+          <t>22/05/2020</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Recovery below target on the first plate</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>I. Alvarado</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>RED run, repeat</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>15/05/2020</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Revised labware, recovery checked</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>I. Alvarado</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
+          <t>Final result tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Dr B. Rowcroft</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Reviewed by</t>
+          <t>Outcome</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Dr R. Deshmukh</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>22/05/2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Outcome</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Rennelwick prioritised the less bound amides for permeability work after the initial stability ranking proved consistent.</t>
         </is>
@@ -760,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -775,208 +732,108 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Assay</t>
+          <t>Assay / record</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Control / status</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Recovery check</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Note</t>
+          <t>Source record</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Microsomes</t>
+          <t>HLM/RLM stability</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MS-01</t>
+          <t>Verapamil and diltiazem within historical range</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Verapamil</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Human and rat in parallel</t>
+          <t>Original microsomal run sheets</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Microsomes</t>
+          <t>RED PPB</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>MS-02</t>
+          <t>Warfarin binding control</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Verapamil</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Repeat of three compounds with flat t½</t>
+          <t>Original dialysis run sheets</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>Sample cards</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>RED-01</t>
+          <t>B-ACC-2020-02338</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Propranolol</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Below target</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Recovery low on both sides of the dialysis cell</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>RED-02</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Propranolol</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Within target</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Labware changed to the low-binding plate</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Acceptance follows the study plan. RED-01 is kept on the file and excluded from the reported values; the repeat run replaces it in full.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Plate acceptance: microsome runs accepted; RED-02 accepted as the reportable plate.</t>
+          <t>Test-lot and handling records</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Binding recovery</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Recovery is reported alongside each binding result.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Original dialysis recovery records</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Plate acceptance</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Consult the original run sheets for plate-level checks.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Result tables do not specify plate allocation.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A7:G7"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -1480,7 +1337,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reportable plate RED-02 only. Unbound fraction is 100 minus % bound. Recovery is shown beside each record and was not corrected.</t>
+          <t>Bound and unbound percentages are reported at different precision; use the recorded unbound value rather than subtracting the rounded bound percentage. Recovery is shown for each compound.</t>
         </is>
       </c>
     </row>

</xml_diff>